<commit_message>
Framework, bitness, BRS version and main form caption updates
</commit_message>
<xml_diff>
--- a/CIF's.xlsx
+++ b/CIF's.xlsx
@@ -19377,8 +19377,8 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101001DFC92230626B54BBA18E48D9F9C68C7" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="f51eaf075755f83ede16354eb286e806">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="66ed17d7-f49c-4dc0-8bf0-446da7d6a21d" xmlns:ns3="ce8fab19-0f33-4450-bfcf-1d15a21b7264" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="f55cec3504a03a4653fc7c0b4b32274d" ns2:_="" ns3:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101001DFC92230626B54BBA18E48D9F9C68C7" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1cc46b72d98582464f6d3dfe67d3566f">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="66ed17d7-f49c-4dc0-8bf0-446da7d6a21d" xmlns:ns3="ce8fab19-0f33-4450-bfcf-1d15a21b7264" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="99438d637b8cea183eae89c30a2c1f5d" ns2:_="" ns3:_="">
     <xsd:import namespace="66ed17d7-f49c-4dc0-8bf0-446da7d6a21d"/>
     <xsd:import namespace="ce8fab19-0f33-4450-bfcf-1d15a21b7264"/>
     <xsd:element name="properties">
@@ -19652,7 +19652,7 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DE752621-DE8B-49A3-A48E-954863F5C975}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9ECF8415-7AD3-47B0-90B4-6B53266EC65F}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>